<commit_message>
feat: generate full-year demo dataset
</commit_message>
<xml_diff>
--- a/data/dnb/2025-01.xlsx
+++ b/data/dnb/2025-01.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,72 +453,72 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45716</v>
+        <v>45681</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SPOTIFY AB</t>
+          <t>MENY BOGSTADVEIEN</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>129</v>
+        <v>684.55</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45714</v>
+        <v>45676</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NETFLIX.COM</t>
+          <t>VINMONOPOLET OSLO S</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>179</v>
+        <v>459</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45712</v>
+        <v>45674</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KIWI MAJORSTUEN</t>
+          <t>POWER STORO</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>456.8</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45710</v>
+        <v>45670</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>REMA 1000 TORSHOV</t>
+          <t>NETFLIX.COM</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>892.3</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45708</v>
+        <v>45668</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>VINMONOPOLET OSLO S</t>
+          <t>REMA 1000 TORSHOV</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>675</v>
+        <v>738.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45706</v>
+        <v>45665</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -526,12 +526,12 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45703</v>
+        <v>45663</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -544,79 +544,27 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45700</v>
+        <v>45661</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAS EUROBONUS</t>
+          <t>KIWI MAJORSTUEN</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2890</v>
+        <v>489.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45698</v>
+        <v>45659</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MENY BOGSTADVEIEN</t>
+          <t>XXL SPORT ALNA</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>567.45</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>45696</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>POWER STORO</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>1299</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>45693</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>COOP EXTRA GRØNLAND</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>723.9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>45691</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Innbetaling</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>45689</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>XXL SPORT ALNA</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
         <v>1499</v>
       </c>
     </row>

</xml_diff>